<commit_message>
fix: preserve spreadsheet data with compact IO validation
</commit_message>
<xml_diff>
--- a/data/example_output/rejected.xlsx
+++ b/data/example_output/rejected.xlsx
@@ -473,6 +473,11 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>__extra_values</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>__issue</t>
         </is>
       </c>
@@ -521,7 +526,8 @@
           <t>64</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr">
         <is>
           <t>missing_id</t>
         </is>
@@ -577,7 +583,8 @@
           <t>65</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
         <is>
           <t>invalid_number_latitude</t>
         </is>
@@ -627,7 +634,8 @@
           <t>66</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
         <is>
           <t>missing_time</t>
         </is>
@@ -677,7 +685,8 @@
           <t>64</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr">
         <is>
           <t>missing_id</t>
         </is>
@@ -733,7 +742,8 @@
           <t>65</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr">
         <is>
           <t>invalid_number_latitude</t>
         </is>
@@ -783,7 +793,8 @@
           <t>66</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
         <is>
           <t>missing_time</t>
         </is>
@@ -833,7 +844,8 @@
           <t>64</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr">
         <is>
           <t>missing_id</t>
         </is>
@@ -889,7 +901,8 @@
           <t>65</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr">
         <is>
           <t>invalid_number_latitude</t>
         </is>
@@ -939,7 +952,8 @@
           <t>66</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
         <is>
           <t>missing_time</t>
         </is>

</xml_diff>